<commit_message>
update naming_conventions regarding CVP/MITTE , inspect canton ZH uebrige, inspect canton uri freie listen
</commit_message>
<xml_diff>
--- a/data/datasets/schwyz/SZ_24_kantonsprotokoll.xlsx
+++ b/data/datasets/schwyz/SZ_24_kantonsprotokoll.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Moritz\Desktop\semester_6\BA\BA_Thesis\data\datasets\schwyz\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Moritz\Desktop\HSG\BA\BA_Thesis\data\datasets\schwyz\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="8_{6B12A3E3-1AAD-4160-A307-C80FB4B801D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="25440" windowHeight="15270" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Stat" sheetId="1" r:id="rId1"/>
@@ -630,10 +630,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="4">
-    <numFmt numFmtId="166" formatCode="\@"/>
-    <numFmt numFmtId="170" formatCode="#,##0.00_ ;\-#,##0.00\ "/>
-    <numFmt numFmtId="171" formatCode="0.0000"/>
-    <numFmt numFmtId="172" formatCode="#,##0.0000"/>
+    <numFmt numFmtId="164" formatCode="\@"/>
+    <numFmt numFmtId="165" formatCode="#,##0.00_ ;\-#,##0.00\ "/>
+    <numFmt numFmtId="166" formatCode="0.0000"/>
+    <numFmt numFmtId="167" formatCode="#,##0.0000"/>
   </numFmts>
   <fonts count="50" x14ac:knownFonts="1">
     <font>
@@ -1464,7 +1464,7 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="170" fontId="12" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="12" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="13" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1476,7 +1476,7 @@
     <xf numFmtId="3" fontId="15" fillId="4" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="170" fontId="16" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="16" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="3" fontId="17" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1488,7 +1488,7 @@
     <xf numFmtId="3" fontId="19" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="171" fontId="20" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="20" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="28" fillId="12" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1504,18 +1504,18 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="37" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="172" fontId="38" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="38" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1"/>
-    <xf numFmtId="166" fontId="41" fillId="17" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="41" fillId="17" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="166" fontId="42" fillId="18" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="42" fillId="18" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="166" fontId="43" fillId="19" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="43" fillId="19" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="44" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1534,29 +1534,19 @@
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="49" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="172" fontId="38" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="15" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="26" fillId="10" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="171" fontId="20" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="27" fillId="11" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="34" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="5" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1580,20 +1570,30 @@
     <xf numFmtId="3" fontId="25" fillId="9" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="10" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="31" fillId="15" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="11" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="167" fontId="38" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="172" fontId="34" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="20" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="39" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -1601,7 +1601,7 @@
     <xf numFmtId="0" fontId="40" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="42" fillId="18" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="42" fillId="18" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
   </cellXfs>
@@ -1962,20 +1962,20 @@
       </c>
     </row>
     <row r="2" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="34" t="s">
+      <c r="A2" s="53" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="35"/>
-      <c r="C2" s="35"/>
-      <c r="D2" s="35"/>
+      <c r="B2" s="48"/>
+      <c r="C2" s="48"/>
+      <c r="D2" s="48"/>
     </row>
     <row r="3" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="36" t="s">
+      <c r="A3" s="54" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="35"/>
-      <c r="C3" s="35"/>
-      <c r="D3" s="35"/>
+      <c r="B3" s="48"/>
+      <c r="C3" s="48"/>
+      <c r="D3" s="48"/>
     </row>
     <row r="4" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="5" spans="1:4" ht="21" customHeight="1" x14ac:dyDescent="0.3">
@@ -2264,52 +2264,52 @@
       </c>
     </row>
     <row r="2" spans="1:20" ht="50" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="37" t="s">
+      <c r="A2" s="51" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="35"/>
-      <c r="C2" s="35"/>
-      <c r="D2" s="35"/>
-      <c r="E2" s="35"/>
-      <c r="F2" s="35"/>
-      <c r="G2" s="35"/>
-      <c r="H2" s="35"/>
-      <c r="I2" s="35"/>
-      <c r="J2" s="35"/>
-      <c r="K2" s="35"/>
-      <c r="L2" s="35"/>
-      <c r="M2" s="35"/>
-      <c r="N2" s="35"/>
-      <c r="O2" s="35"/>
-      <c r="P2" s="35"/>
-      <c r="Q2" s="35"/>
-      <c r="R2" s="35"/>
-      <c r="S2" s="35"/>
-      <c r="T2" s="35"/>
+      <c r="B2" s="48"/>
+      <c r="C2" s="48"/>
+      <c r="D2" s="48"/>
+      <c r="E2" s="48"/>
+      <c r="F2" s="48"/>
+      <c r="G2" s="48"/>
+      <c r="H2" s="48"/>
+      <c r="I2" s="48"/>
+      <c r="J2" s="48"/>
+      <c r="K2" s="48"/>
+      <c r="L2" s="48"/>
+      <c r="M2" s="48"/>
+      <c r="N2" s="48"/>
+      <c r="O2" s="48"/>
+      <c r="P2" s="48"/>
+      <c r="Q2" s="48"/>
+      <c r="R2" s="48"/>
+      <c r="S2" s="48"/>
+      <c r="T2" s="48"/>
     </row>
     <row r="3" spans="1:20" ht="25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="38" t="s">
+      <c r="A3" s="52" t="s">
         <v>12</v>
       </c>
-      <c r="B3" s="35"/>
-      <c r="C3" s="35"/>
-      <c r="D3" s="35"/>
-      <c r="E3" s="35"/>
-      <c r="F3" s="35"/>
-      <c r="G3" s="35"/>
-      <c r="H3" s="35"/>
-      <c r="I3" s="35"/>
-      <c r="J3" s="35"/>
-      <c r="K3" s="35"/>
-      <c r="L3" s="35"/>
-      <c r="M3" s="35"/>
-      <c r="N3" s="35"/>
-      <c r="O3" s="35"/>
-      <c r="P3" s="35"/>
-      <c r="Q3" s="35"/>
-      <c r="R3" s="35"/>
-      <c r="S3" s="35"/>
-      <c r="T3" s="35"/>
+      <c r="B3" s="48"/>
+      <c r="C3" s="48"/>
+      <c r="D3" s="48"/>
+      <c r="E3" s="48"/>
+      <c r="F3" s="48"/>
+      <c r="G3" s="48"/>
+      <c r="H3" s="48"/>
+      <c r="I3" s="48"/>
+      <c r="J3" s="48"/>
+      <c r="K3" s="48"/>
+      <c r="L3" s="48"/>
+      <c r="M3" s="48"/>
+      <c r="N3" s="48"/>
+      <c r="O3" s="48"/>
+      <c r="P3" s="48"/>
+      <c r="Q3" s="48"/>
+      <c r="R3" s="48"/>
+      <c r="S3" s="48"/>
+      <c r="T3" s="48"/>
     </row>
     <row r="4" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
@@ -2436,149 +2436,149 @@
       </c>
     </row>
     <row r="6" spans="1:20" ht="13" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="43" t="s">
+      <c r="A6" s="39" t="s">
         <v>13</v>
       </c>
-      <c r="B6" s="43" t="s">
-        <v>195</v>
-      </c>
-      <c r="C6" s="46" t="s">
+      <c r="B6" s="39" t="s">
+        <v>195</v>
+      </c>
+      <c r="C6" s="42" t="s">
         <v>14</v>
       </c>
-      <c r="D6" s="46" t="s">
+      <c r="D6" s="42" t="s">
         <v>15</v>
       </c>
-      <c r="E6" s="47" t="s">
+      <c r="E6" s="43" t="s">
         <v>16</v>
       </c>
-      <c r="F6" s="48" t="s">
+      <c r="F6" s="44" t="s">
         <v>17</v>
       </c>
-      <c r="G6" s="49" t="s">
+      <c r="G6" s="45" t="s">
         <v>18</v>
       </c>
-      <c r="H6" s="50" t="s">
+      <c r="H6" s="34" t="s">
         <v>19</v>
       </c>
-      <c r="I6" s="50" t="s">
+      <c r="I6" s="34" t="s">
         <v>15</v>
       </c>
-      <c r="J6" s="50" t="s">
+      <c r="J6" s="34" t="s">
         <v>20</v>
       </c>
-      <c r="K6" s="50" t="s">
+      <c r="K6" s="34" t="s">
         <v>21</v>
       </c>
-      <c r="L6" s="50" t="s">
+      <c r="L6" s="34" t="s">
         <v>15</v>
       </c>
-      <c r="M6" s="50" t="s">
+      <c r="M6" s="34" t="s">
         <v>20</v>
       </c>
-      <c r="N6" s="50" t="s">
+      <c r="N6" s="34" t="s">
         <v>22</v>
       </c>
-      <c r="O6" s="50" t="s">
+      <c r="O6" s="34" t="s">
         <v>15</v>
       </c>
-      <c r="P6" s="50" t="s">
+      <c r="P6" s="34" t="s">
         <v>20</v>
       </c>
-      <c r="Q6" s="50" t="s">
+      <c r="Q6" s="34" t="s">
         <v>23</v>
       </c>
-      <c r="R6" s="50" t="s">
+      <c r="R6" s="34" t="s">
         <v>15</v>
       </c>
-      <c r="S6" s="50" t="s">
+      <c r="S6" s="34" t="s">
         <v>20</v>
       </c>
-      <c r="T6" s="41" t="s">
+      <c r="T6" s="46" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="7" spans="1:20" ht="13" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="43" t="s">
-        <v>195</v>
-      </c>
-      <c r="B7" s="43" t="s">
-        <v>195</v>
-      </c>
-      <c r="C7" s="46" t="s">
-        <v>195</v>
-      </c>
-      <c r="D7" s="46" t="s">
-        <v>195</v>
-      </c>
-      <c r="E7" s="47" t="s">
-        <v>195</v>
-      </c>
-      <c r="F7" s="48" t="s">
-        <v>195</v>
-      </c>
-      <c r="G7" s="49" t="s">
-        <v>195</v>
-      </c>
-      <c r="H7" s="51" t="s">
+      <c r="A7" s="39" t="s">
+        <v>195</v>
+      </c>
+      <c r="B7" s="39" t="s">
+        <v>195</v>
+      </c>
+      <c r="C7" s="42" t="s">
+        <v>195</v>
+      </c>
+      <c r="D7" s="42" t="s">
+        <v>195</v>
+      </c>
+      <c r="E7" s="43" t="s">
+        <v>195</v>
+      </c>
+      <c r="F7" s="44" t="s">
+        <v>195</v>
+      </c>
+      <c r="G7" s="45" t="s">
+        <v>195</v>
+      </c>
+      <c r="H7" s="35" t="s">
         <v>25</v>
       </c>
-      <c r="I7" s="51" t="s">
-        <v>195</v>
-      </c>
-      <c r="J7" s="51" t="s">
-        <v>195</v>
-      </c>
-      <c r="K7" s="51" t="s">
+      <c r="I7" s="35" t="s">
+        <v>195</v>
+      </c>
+      <c r="J7" s="35" t="s">
+        <v>195</v>
+      </c>
+      <c r="K7" s="35" t="s">
         <v>26</v>
       </c>
-      <c r="L7" s="51" t="s">
-        <v>195</v>
-      </c>
-      <c r="M7" s="51" t="s">
-        <v>195</v>
-      </c>
-      <c r="N7" s="51" t="s">
+      <c r="L7" s="35" t="s">
+        <v>195</v>
+      </c>
+      <c r="M7" s="35" t="s">
+        <v>195</v>
+      </c>
+      <c r="N7" s="35" t="s">
         <v>27</v>
       </c>
-      <c r="O7" s="51" t="s">
-        <v>195</v>
-      </c>
-      <c r="P7" s="51" t="s">
-        <v>195</v>
-      </c>
-      <c r="Q7" s="51" t="s">
+      <c r="O7" s="35" t="s">
+        <v>195</v>
+      </c>
+      <c r="P7" s="35" t="s">
+        <v>195</v>
+      </c>
+      <c r="Q7" s="35" t="s">
         <v>28</v>
       </c>
-      <c r="R7" s="51" t="s">
-        <v>195</v>
-      </c>
-      <c r="S7" s="51" t="s">
-        <v>195</v>
-      </c>
-      <c r="T7" s="41" t="s">
+      <c r="R7" s="35" t="s">
+        <v>195</v>
+      </c>
+      <c r="S7" s="35" t="s">
+        <v>195</v>
+      </c>
+      <c r="T7" s="46" t="s">
         <v>195</v>
       </c>
     </row>
     <row r="8" spans="1:20" ht="22" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="43" t="s">
+      <c r="A8" s="39" t="s">
         <v>13</v>
       </c>
-      <c r="B8" s="43" t="s">
-        <v>195</v>
-      </c>
-      <c r="C8" s="46" t="s">
+      <c r="B8" s="39" t="s">
+        <v>195</v>
+      </c>
+      <c r="C8" s="42" t="s">
         <v>14</v>
       </c>
-      <c r="D8" s="46" t="s">
+      <c r="D8" s="42" t="s">
         <v>15</v>
       </c>
-      <c r="E8" s="47" t="s">
+      <c r="E8" s="43" t="s">
         <v>16</v>
       </c>
-      <c r="F8" s="48" t="s">
+      <c r="F8" s="44" t="s">
         <v>17</v>
       </c>
-      <c r="G8" s="49" t="s">
+      <c r="G8" s="45" t="s">
         <v>18</v>
       </c>
       <c r="H8" s="17" t="s">
@@ -2617,7 +2617,7 @@
       <c r="S8" s="19" t="s">
         <v>20</v>
       </c>
-      <c r="T8" s="41" t="s">
+      <c r="T8" s="46" t="s">
         <v>24</v>
       </c>
     </row>
@@ -2968,41 +2968,41 @@
       <c r="B15" s="20"/>
       <c r="C15" s="20"/>
       <c r="D15" s="20"/>
-      <c r="E15" s="44" t="s">
+      <c r="E15" s="40" t="s">
         <v>43</v>
       </c>
-      <c r="F15" s="44"/>
-      <c r="G15" s="45"/>
-      <c r="H15" s="52">
+      <c r="F15" s="40"/>
+      <c r="G15" s="41"/>
+      <c r="H15" s="36">
         <v>5622.4444444444443</v>
       </c>
-      <c r="I15" s="53"/>
-      <c r="J15" s="54"/>
-      <c r="K15" s="52">
+      <c r="I15" s="37"/>
+      <c r="J15" s="38"/>
+      <c r="K15" s="36">
         <v>3050.4285714285716</v>
       </c>
-      <c r="L15" s="53"/>
-      <c r="M15" s="54"/>
-      <c r="N15" s="52">
+      <c r="L15" s="37"/>
+      <c r="M15" s="38"/>
+      <c r="N15" s="36">
         <v>3343.0500000000006</v>
       </c>
-      <c r="O15" s="53"/>
-      <c r="P15" s="54"/>
-      <c r="Q15" s="52">
+      <c r="O15" s="37"/>
+      <c r="P15" s="38"/>
+      <c r="Q15" s="36">
         <v>1603.5</v>
       </c>
-      <c r="R15" s="53"/>
-      <c r="S15" s="54"/>
+      <c r="R15" s="37"/>
+      <c r="S15" s="38"/>
     </row>
     <row r="16" spans="1:20" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="21" t="s">
         <v>44</v>
       </c>
-      <c r="D16" s="39">
+      <c r="D16" s="47">
         <v>543.82320238095235</v>
       </c>
-      <c r="E16" s="35"/>
-      <c r="F16" s="35"/>
+      <c r="E16" s="48"/>
+      <c r="F16" s="48"/>
       <c r="G16" s="21" t="s">
         <v>45</v>
       </c>
@@ -3135,149 +3135,149 @@
       </c>
     </row>
     <row r="19" spans="1:20" ht="13" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="43" t="s">
+      <c r="A19" s="39" t="s">
         <v>13</v>
       </c>
-      <c r="B19" s="43" t="s">
-        <v>195</v>
-      </c>
-      <c r="C19" s="46" t="s">
+      <c r="B19" s="39" t="s">
+        <v>195</v>
+      </c>
+      <c r="C19" s="42" t="s">
         <v>14</v>
       </c>
-      <c r="D19" s="46" t="s">
+      <c r="D19" s="42" t="s">
         <v>15</v>
       </c>
-      <c r="E19" s="47" t="s">
+      <c r="E19" s="43" t="s">
         <v>16</v>
       </c>
-      <c r="F19" s="48" t="s">
+      <c r="F19" s="44" t="s">
         <v>17</v>
       </c>
-      <c r="G19" s="49" t="s">
+      <c r="G19" s="45" t="s">
         <v>18</v>
       </c>
-      <c r="H19" s="50" t="s">
+      <c r="H19" s="34" t="s">
         <v>46</v>
       </c>
-      <c r="I19" s="50" t="s">
+      <c r="I19" s="34" t="s">
         <v>15</v>
       </c>
-      <c r="J19" s="50" t="s">
+      <c r="J19" s="34" t="s">
         <v>20</v>
       </c>
-      <c r="K19" s="50" t="s">
+      <c r="K19" s="34" t="s">
         <v>47</v>
       </c>
-      <c r="L19" s="50" t="s">
+      <c r="L19" s="34" t="s">
         <v>15</v>
       </c>
-      <c r="M19" s="50" t="s">
+      <c r="M19" s="34" t="s">
         <v>20</v>
       </c>
-      <c r="N19" s="50" t="s">
+      <c r="N19" s="34" t="s">
         <v>48</v>
       </c>
-      <c r="O19" s="50" t="s">
+      <c r="O19" s="34" t="s">
         <v>15</v>
       </c>
-      <c r="P19" s="50" t="s">
+      <c r="P19" s="34" t="s">
         <v>20</v>
       </c>
-      <c r="Q19" s="50" t="s">
+      <c r="Q19" s="34" t="s">
         <v>49</v>
       </c>
-      <c r="R19" s="50" t="s">
+      <c r="R19" s="34" t="s">
         <v>15</v>
       </c>
-      <c r="S19" s="50" t="s">
+      <c r="S19" s="34" t="s">
         <v>20</v>
       </c>
-      <c r="T19" s="41" t="s">
+      <c r="T19" s="46" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="20" spans="1:20" ht="13" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="43" t="s">
-        <v>195</v>
-      </c>
-      <c r="B20" s="43" t="s">
-        <v>195</v>
-      </c>
-      <c r="C20" s="46" t="s">
-        <v>195</v>
-      </c>
-      <c r="D20" s="46" t="s">
-        <v>195</v>
-      </c>
-      <c r="E20" s="47" t="s">
-        <v>195</v>
-      </c>
-      <c r="F20" s="48" t="s">
-        <v>195</v>
-      </c>
-      <c r="G20" s="49" t="s">
-        <v>195</v>
-      </c>
-      <c r="H20" s="51" t="s">
+      <c r="A20" s="39" t="s">
+        <v>195</v>
+      </c>
+      <c r="B20" s="39" t="s">
+        <v>195</v>
+      </c>
+      <c r="C20" s="42" t="s">
+        <v>195</v>
+      </c>
+      <c r="D20" s="42" t="s">
+        <v>195</v>
+      </c>
+      <c r="E20" s="43" t="s">
+        <v>195</v>
+      </c>
+      <c r="F20" s="44" t="s">
+        <v>195</v>
+      </c>
+      <c r="G20" s="45" t="s">
+        <v>195</v>
+      </c>
+      <c r="H20" s="35" t="s">
         <v>28</v>
       </c>
-      <c r="I20" s="51" t="s">
-        <v>195</v>
-      </c>
-      <c r="J20" s="51" t="s">
-        <v>195</v>
-      </c>
-      <c r="K20" s="51" t="s">
+      <c r="I20" s="35" t="s">
+        <v>195</v>
+      </c>
+      <c r="J20" s="35" t="s">
+        <v>195</v>
+      </c>
+      <c r="K20" s="35" t="s">
         <v>50</v>
       </c>
-      <c r="L20" s="51" t="s">
-        <v>195</v>
-      </c>
-      <c r="M20" s="51" t="s">
-        <v>195</v>
-      </c>
-      <c r="N20" s="51" t="s">
+      <c r="L20" s="35" t="s">
+        <v>195</v>
+      </c>
+      <c r="M20" s="35" t="s">
+        <v>195</v>
+      </c>
+      <c r="N20" s="35" t="s">
         <v>28</v>
       </c>
-      <c r="O20" s="51" t="s">
-        <v>195</v>
-      </c>
-      <c r="P20" s="51" t="s">
-        <v>195</v>
-      </c>
-      <c r="Q20" s="51" t="s">
+      <c r="O20" s="35" t="s">
+        <v>195</v>
+      </c>
+      <c r="P20" s="35" t="s">
+        <v>195</v>
+      </c>
+      <c r="Q20" s="35" t="s">
         <v>50</v>
       </c>
-      <c r="R20" s="51" t="s">
-        <v>195</v>
-      </c>
-      <c r="S20" s="51" t="s">
-        <v>195</v>
-      </c>
-      <c r="T20" s="41" t="s">
+      <c r="R20" s="35" t="s">
+        <v>195</v>
+      </c>
+      <c r="S20" s="35" t="s">
+        <v>195</v>
+      </c>
+      <c r="T20" s="46" t="s">
         <v>195</v>
       </c>
     </row>
     <row r="21" spans="1:20" ht="22" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="43" t="s">
+      <c r="A21" s="39" t="s">
         <v>13</v>
       </c>
-      <c r="B21" s="43" t="s">
-        <v>195</v>
-      </c>
-      <c r="C21" s="46" t="s">
+      <c r="B21" s="39" t="s">
+        <v>195</v>
+      </c>
+      <c r="C21" s="42" t="s">
         <v>14</v>
       </c>
-      <c r="D21" s="46" t="s">
+      <c r="D21" s="42" t="s">
         <v>15</v>
       </c>
-      <c r="E21" s="47" t="s">
+      <c r="E21" s="43" t="s">
         <v>16</v>
       </c>
-      <c r="F21" s="48" t="s">
+      <c r="F21" s="44" t="s">
         <v>17</v>
       </c>
-      <c r="G21" s="49" t="s">
+      <c r="G21" s="45" t="s">
         <v>18</v>
       </c>
       <c r="H21" s="17" t="s">
@@ -3316,7 +3316,7 @@
       <c r="S21" s="19" t="s">
         <v>20</v>
       </c>
-      <c r="T21" s="41" t="s">
+      <c r="T21" s="46" t="s">
         <v>24</v>
       </c>
     </row>
@@ -3633,41 +3633,41 @@
       <c r="B28" s="20"/>
       <c r="C28" s="20"/>
       <c r="D28" s="20"/>
-      <c r="E28" s="44" t="s">
+      <c r="E28" s="40" t="s">
         <v>43</v>
       </c>
-      <c r="F28" s="44"/>
-      <c r="G28" s="45"/>
-      <c r="H28" s="52">
+      <c r="F28" s="40"/>
+      <c r="G28" s="41"/>
+      <c r="H28" s="36">
         <v>1764.5625</v>
       </c>
-      <c r="I28" s="53"/>
-      <c r="J28" s="54"/>
-      <c r="K28" s="52">
+      <c r="I28" s="37"/>
+      <c r="J28" s="38"/>
+      <c r="K28" s="36">
         <v>834</v>
       </c>
-      <c r="L28" s="53"/>
-      <c r="M28" s="54"/>
-      <c r="N28" s="52">
+      <c r="L28" s="37"/>
+      <c r="M28" s="38"/>
+      <c r="N28" s="36">
         <v>1055</v>
       </c>
-      <c r="O28" s="53"/>
-      <c r="P28" s="54"/>
-      <c r="Q28" s="52">
+      <c r="O28" s="37"/>
+      <c r="P28" s="38"/>
+      <c r="Q28" s="36">
         <v>464</v>
       </c>
-      <c r="R28" s="53"/>
-      <c r="S28" s="54"/>
+      <c r="R28" s="37"/>
+      <c r="S28" s="38"/>
     </row>
     <row r="29" spans="1:20" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="21" t="s">
         <v>44</v>
       </c>
-      <c r="D29" s="39">
+      <c r="D29" s="47">
         <v>543.82320238095235</v>
       </c>
-      <c r="E29" s="35"/>
-      <c r="F29" s="35"/>
+      <c r="E29" s="48"/>
+      <c r="F29" s="48"/>
       <c r="G29" s="21" t="s">
         <v>45</v>
       </c>
@@ -3800,149 +3800,149 @@
       </c>
     </row>
     <row r="32" spans="1:20" ht="13" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="43" t="s">
+      <c r="A32" s="39" t="s">
         <v>13</v>
       </c>
-      <c r="B32" s="43" t="s">
-        <v>195</v>
-      </c>
-      <c r="C32" s="46" t="s">
+      <c r="B32" s="39" t="s">
+        <v>195</v>
+      </c>
+      <c r="C32" s="42" t="s">
         <v>14</v>
       </c>
-      <c r="D32" s="46" t="s">
+      <c r="D32" s="42" t="s">
         <v>15</v>
       </c>
-      <c r="E32" s="47" t="s">
+      <c r="E32" s="43" t="s">
         <v>16</v>
       </c>
-      <c r="F32" s="48" t="s">
+      <c r="F32" s="44" t="s">
         <v>17</v>
       </c>
-      <c r="G32" s="49" t="s">
+      <c r="G32" s="45" t="s">
         <v>18</v>
       </c>
-      <c r="H32" s="50" t="s">
+      <c r="H32" s="34" t="s">
         <v>51</v>
       </c>
-      <c r="I32" s="50" t="s">
+      <c r="I32" s="34" t="s">
         <v>15</v>
       </c>
-      <c r="J32" s="50" t="s">
+      <c r="J32" s="34" t="s">
         <v>20</v>
       </c>
-      <c r="K32" s="50" t="s">
+      <c r="K32" s="34" t="s">
         <v>52</v>
       </c>
-      <c r="L32" s="50" t="s">
+      <c r="L32" s="34" t="s">
         <v>15</v>
       </c>
-      <c r="M32" s="50" t="s">
+      <c r="M32" s="34" t="s">
         <v>20</v>
       </c>
-      <c r="N32" s="50" t="s">
+      <c r="N32" s="34" t="s">
         <v>53</v>
       </c>
-      <c r="O32" s="50" t="s">
+      <c r="O32" s="34" t="s">
         <v>15</v>
       </c>
-      <c r="P32" s="50" t="s">
+      <c r="P32" s="34" t="s">
         <v>20</v>
       </c>
-      <c r="Q32" s="50" t="s">
+      <c r="Q32" s="34" t="s">
         <v>54</v>
       </c>
-      <c r="R32" s="50" t="s">
+      <c r="R32" s="34" t="s">
         <v>15</v>
       </c>
-      <c r="S32" s="50" t="s">
+      <c r="S32" s="34" t="s">
         <v>20</v>
       </c>
-      <c r="T32" s="41" t="s">
+      <c r="T32" s="46" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="33" spans="1:20" ht="13" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="43" t="s">
-        <v>195</v>
-      </c>
-      <c r="B33" s="43" t="s">
-        <v>195</v>
-      </c>
-      <c r="C33" s="46" t="s">
-        <v>195</v>
-      </c>
-      <c r="D33" s="46" t="s">
-        <v>195</v>
-      </c>
-      <c r="E33" s="47" t="s">
-        <v>195</v>
-      </c>
-      <c r="F33" s="48" t="s">
-        <v>195</v>
-      </c>
-      <c r="G33" s="49" t="s">
-        <v>195</v>
-      </c>
-      <c r="H33" s="51" t="s">
+      <c r="A33" s="39" t="s">
+        <v>195</v>
+      </c>
+      <c r="B33" s="39" t="s">
+        <v>195</v>
+      </c>
+      <c r="C33" s="42" t="s">
+        <v>195</v>
+      </c>
+      <c r="D33" s="42" t="s">
+        <v>195</v>
+      </c>
+      <c r="E33" s="43" t="s">
+        <v>195</v>
+      </c>
+      <c r="F33" s="44" t="s">
+        <v>195</v>
+      </c>
+      <c r="G33" s="45" t="s">
+        <v>195</v>
+      </c>
+      <c r="H33" s="35" t="s">
         <v>28</v>
       </c>
-      <c r="I33" s="51" t="s">
-        <v>195</v>
-      </c>
-      <c r="J33" s="51" t="s">
-        <v>195</v>
-      </c>
-      <c r="K33" s="51" t="s">
+      <c r="I33" s="35" t="s">
+        <v>195</v>
+      </c>
+      <c r="J33" s="35" t="s">
+        <v>195</v>
+      </c>
+      <c r="K33" s="35" t="s">
         <v>50</v>
       </c>
-      <c r="L33" s="51" t="s">
-        <v>195</v>
-      </c>
-      <c r="M33" s="51" t="s">
-        <v>195</v>
-      </c>
-      <c r="N33" s="51" t="s">
+      <c r="L33" s="35" t="s">
+        <v>195</v>
+      </c>
+      <c r="M33" s="35" t="s">
+        <v>195</v>
+      </c>
+      <c r="N33" s="35" t="s">
         <v>50</v>
       </c>
-      <c r="O33" s="51" t="s">
-        <v>195</v>
-      </c>
-      <c r="P33" s="51" t="s">
-        <v>195</v>
-      </c>
-      <c r="Q33" s="51" t="s">
+      <c r="O33" s="35" t="s">
+        <v>195</v>
+      </c>
+      <c r="P33" s="35" t="s">
+        <v>195</v>
+      </c>
+      <c r="Q33" s="35" t="s">
         <v>50</v>
       </c>
-      <c r="R33" s="51" t="s">
-        <v>195</v>
-      </c>
-      <c r="S33" s="51" t="s">
-        <v>195</v>
-      </c>
-      <c r="T33" s="41" t="s">
+      <c r="R33" s="35" t="s">
+        <v>195</v>
+      </c>
+      <c r="S33" s="35" t="s">
+        <v>195</v>
+      </c>
+      <c r="T33" s="46" t="s">
         <v>195</v>
       </c>
     </row>
     <row r="34" spans="1:20" ht="22" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="43" t="s">
+      <c r="A34" s="39" t="s">
         <v>13</v>
       </c>
-      <c r="B34" s="43" t="s">
-        <v>195</v>
-      </c>
-      <c r="C34" s="46" t="s">
+      <c r="B34" s="39" t="s">
+        <v>195</v>
+      </c>
+      <c r="C34" s="42" t="s">
         <v>14</v>
       </c>
-      <c r="D34" s="46" t="s">
+      <c r="D34" s="42" t="s">
         <v>15</v>
       </c>
-      <c r="E34" s="47" t="s">
+      <c r="E34" s="43" t="s">
         <v>16</v>
       </c>
-      <c r="F34" s="48" t="s">
+      <c r="F34" s="44" t="s">
         <v>17</v>
       </c>
-      <c r="G34" s="49" t="s">
+      <c r="G34" s="45" t="s">
         <v>18</v>
       </c>
       <c r="H34" s="17" t="s">
@@ -3981,7 +3981,7 @@
       <c r="S34" s="19" t="s">
         <v>20</v>
       </c>
-      <c r="T34" s="41" t="s">
+      <c r="T34" s="46" t="s">
         <v>24</v>
       </c>
     </row>
@@ -4288,41 +4288,41 @@
       <c r="B41" s="20"/>
       <c r="C41" s="20"/>
       <c r="D41" s="20"/>
-      <c r="E41" s="44" t="s">
+      <c r="E41" s="40" t="s">
         <v>43</v>
       </c>
-      <c r="F41" s="44"/>
-      <c r="G41" s="45"/>
-      <c r="H41" s="52">
+      <c r="F41" s="40"/>
+      <c r="G41" s="41"/>
+      <c r="H41" s="36">
         <v>1038</v>
       </c>
-      <c r="I41" s="53"/>
-      <c r="J41" s="54"/>
-      <c r="K41" s="52">
+      <c r="I41" s="37"/>
+      <c r="J41" s="38"/>
+      <c r="K41" s="36">
         <v>473</v>
       </c>
-      <c r="L41" s="53"/>
-      <c r="M41" s="54"/>
-      <c r="N41" s="52">
+      <c r="L41" s="37"/>
+      <c r="M41" s="38"/>
+      <c r="N41" s="36">
         <v>420</v>
       </c>
-      <c r="O41" s="53"/>
-      <c r="P41" s="54"/>
-      <c r="Q41" s="52">
+      <c r="O41" s="37"/>
+      <c r="P41" s="38"/>
+      <c r="Q41" s="36">
         <v>494</v>
       </c>
-      <c r="R41" s="53"/>
-      <c r="S41" s="54"/>
+      <c r="R41" s="37"/>
+      <c r="S41" s="38"/>
     </row>
     <row r="42" spans="1:20" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42" s="21" t="s">
         <v>44</v>
       </c>
-      <c r="D42" s="39">
+      <c r="D42" s="47">
         <v>543.82320238095235</v>
       </c>
-      <c r="E42" s="35"/>
-      <c r="F42" s="35"/>
+      <c r="E42" s="48"/>
+      <c r="F42" s="48"/>
       <c r="G42" s="21" t="s">
         <v>45</v>
       </c>
@@ -4641,149 +4641,149 @@
       </c>
     </row>
     <row r="48" spans="1:20" ht="13" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A48" s="43" t="s">
+      <c r="A48" s="39" t="s">
         <v>13</v>
       </c>
-      <c r="B48" s="43" t="s">
-        <v>195</v>
-      </c>
-      <c r="C48" s="46" t="s">
+      <c r="B48" s="39" t="s">
+        <v>195</v>
+      </c>
+      <c r="C48" s="42" t="s">
         <v>14</v>
       </c>
-      <c r="D48" s="46" t="s">
+      <c r="D48" s="42" t="s">
         <v>15</v>
       </c>
-      <c r="E48" s="47" t="s">
+      <c r="E48" s="43" t="s">
         <v>16</v>
       </c>
-      <c r="F48" s="48" t="s">
+      <c r="F48" s="44" t="s">
         <v>17</v>
       </c>
-      <c r="G48" s="49" t="s">
+      <c r="G48" s="45" t="s">
         <v>18</v>
       </c>
-      <c r="H48" s="50" t="s">
+      <c r="H48" s="34" t="s">
         <v>55</v>
       </c>
-      <c r="I48" s="50" t="s">
+      <c r="I48" s="34" t="s">
         <v>15</v>
       </c>
-      <c r="J48" s="50" t="s">
+      <c r="J48" s="34" t="s">
         <v>20</v>
       </c>
-      <c r="K48" s="50" t="s">
+      <c r="K48" s="34" t="s">
         <v>56</v>
       </c>
-      <c r="L48" s="50" t="s">
+      <c r="L48" s="34" t="s">
         <v>15</v>
       </c>
-      <c r="M48" s="50" t="s">
+      <c r="M48" s="34" t="s">
         <v>20</v>
       </c>
-      <c r="N48" s="50" t="s">
+      <c r="N48" s="34" t="s">
         <v>57</v>
       </c>
-      <c r="O48" s="50" t="s">
+      <c r="O48" s="34" t="s">
         <v>15</v>
       </c>
-      <c r="P48" s="50" t="s">
+      <c r="P48" s="34" t="s">
         <v>20</v>
       </c>
-      <c r="Q48" s="50" t="s">
+      <c r="Q48" s="34" t="s">
         <v>58</v>
       </c>
-      <c r="R48" s="50" t="s">
+      <c r="R48" s="34" t="s">
         <v>15</v>
       </c>
-      <c r="S48" s="50" t="s">
+      <c r="S48" s="34" t="s">
         <v>20</v>
       </c>
-      <c r="T48" s="41" t="s">
+      <c r="T48" s="46" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="49" spans="1:20" ht="13" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A49" s="43" t="s">
-        <v>195</v>
-      </c>
-      <c r="B49" s="43" t="s">
-        <v>195</v>
-      </c>
-      <c r="C49" s="46" t="s">
-        <v>195</v>
-      </c>
-      <c r="D49" s="46" t="s">
-        <v>195</v>
-      </c>
-      <c r="E49" s="47" t="s">
-        <v>195</v>
-      </c>
-      <c r="F49" s="48" t="s">
-        <v>195</v>
-      </c>
-      <c r="G49" s="49" t="s">
-        <v>195</v>
-      </c>
-      <c r="H49" s="51" t="s">
+      <c r="A49" s="39" t="s">
+        <v>195</v>
+      </c>
+      <c r="B49" s="39" t="s">
+        <v>195</v>
+      </c>
+      <c r="C49" s="42" t="s">
+        <v>195</v>
+      </c>
+      <c r="D49" s="42" t="s">
+        <v>195</v>
+      </c>
+      <c r="E49" s="43" t="s">
+        <v>195</v>
+      </c>
+      <c r="F49" s="44" t="s">
+        <v>195</v>
+      </c>
+      <c r="G49" s="45" t="s">
+        <v>195</v>
+      </c>
+      <c r="H49" s="35" t="s">
         <v>50</v>
       </c>
-      <c r="I49" s="51" t="s">
-        <v>195</v>
-      </c>
-      <c r="J49" s="51" t="s">
-        <v>195</v>
-      </c>
-      <c r="K49" s="51" t="s">
+      <c r="I49" s="35" t="s">
+        <v>195</v>
+      </c>
+      <c r="J49" s="35" t="s">
+        <v>195</v>
+      </c>
+      <c r="K49" s="35" t="s">
         <v>50</v>
       </c>
-      <c r="L49" s="51" t="s">
-        <v>195</v>
-      </c>
-      <c r="M49" s="51" t="s">
-        <v>195</v>
-      </c>
-      <c r="N49" s="51" t="s">
+      <c r="L49" s="35" t="s">
+        <v>195</v>
+      </c>
+      <c r="M49" s="35" t="s">
+        <v>195</v>
+      </c>
+      <c r="N49" s="35" t="s">
         <v>50</v>
       </c>
-      <c r="O49" s="51" t="s">
-        <v>195</v>
-      </c>
-      <c r="P49" s="51" t="s">
-        <v>195</v>
-      </c>
-      <c r="Q49" s="51" t="s">
+      <c r="O49" s="35" t="s">
+        <v>195</v>
+      </c>
+      <c r="P49" s="35" t="s">
+        <v>195</v>
+      </c>
+      <c r="Q49" s="35" t="s">
         <v>50</v>
       </c>
-      <c r="R49" s="51" t="s">
-        <v>195</v>
-      </c>
-      <c r="S49" s="51" t="s">
-        <v>195</v>
-      </c>
-      <c r="T49" s="41" t="s">
+      <c r="R49" s="35" t="s">
+        <v>195</v>
+      </c>
+      <c r="S49" s="35" t="s">
+        <v>195</v>
+      </c>
+      <c r="T49" s="46" t="s">
         <v>195</v>
       </c>
     </row>
     <row r="50" spans="1:20" ht="22" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="43" t="s">
+      <c r="A50" s="39" t="s">
         <v>13</v>
       </c>
-      <c r="B50" s="43" t="s">
-        <v>195</v>
-      </c>
-      <c r="C50" s="46" t="s">
+      <c r="B50" s="39" t="s">
+        <v>195</v>
+      </c>
+      <c r="C50" s="42" t="s">
         <v>14</v>
       </c>
-      <c r="D50" s="46" t="s">
+      <c r="D50" s="42" t="s">
         <v>15</v>
       </c>
-      <c r="E50" s="47" t="s">
+      <c r="E50" s="43" t="s">
         <v>16</v>
       </c>
-      <c r="F50" s="48" t="s">
+      <c r="F50" s="44" t="s">
         <v>17</v>
       </c>
-      <c r="G50" s="49" t="s">
+      <c r="G50" s="45" t="s">
         <v>18</v>
       </c>
       <c r="H50" s="17" t="s">
@@ -4822,7 +4822,7 @@
       <c r="S50" s="19" t="s">
         <v>20</v>
       </c>
-      <c r="T50" s="41" t="s">
+      <c r="T50" s="46" t="s">
         <v>24</v>
       </c>
     </row>
@@ -5117,41 +5117,41 @@
       <c r="B57" s="20"/>
       <c r="C57" s="20"/>
       <c r="D57" s="20"/>
-      <c r="E57" s="44" t="s">
+      <c r="E57" s="40" t="s">
         <v>43</v>
       </c>
-      <c r="F57" s="44"/>
-      <c r="G57" s="45"/>
-      <c r="H57" s="52">
+      <c r="F57" s="40"/>
+      <c r="G57" s="41"/>
+      <c r="H57" s="36">
         <v>233</v>
       </c>
-      <c r="I57" s="53"/>
-      <c r="J57" s="54"/>
-      <c r="K57" s="52">
+      <c r="I57" s="37"/>
+      <c r="J57" s="38"/>
+      <c r="K57" s="36">
         <v>470</v>
       </c>
-      <c r="L57" s="53"/>
-      <c r="M57" s="54"/>
-      <c r="N57" s="52">
+      <c r="L57" s="37"/>
+      <c r="M57" s="38"/>
+      <c r="N57" s="36">
         <v>39</v>
       </c>
-      <c r="O57" s="53"/>
-      <c r="P57" s="54"/>
-      <c r="Q57" s="52">
+      <c r="O57" s="37"/>
+      <c r="P57" s="38"/>
+      <c r="Q57" s="36">
         <v>658.5</v>
       </c>
-      <c r="R57" s="53"/>
-      <c r="S57" s="54"/>
+      <c r="R57" s="37"/>
+      <c r="S57" s="38"/>
     </row>
     <row r="58" spans="1:20" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A58" s="21" t="s">
         <v>44</v>
       </c>
-      <c r="D58" s="39">
+      <c r="D58" s="47">
         <v>543.82320238095235</v>
       </c>
-      <c r="E58" s="35"/>
-      <c r="F58" s="35"/>
+      <c r="E58" s="48"/>
+      <c r="F58" s="48"/>
       <c r="G58" s="21" t="s">
         <v>45</v>
       </c>
@@ -5284,149 +5284,149 @@
       </c>
     </row>
     <row r="61" spans="1:20" ht="13" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A61" s="43" t="s">
+      <c r="A61" s="39" t="s">
         <v>13</v>
       </c>
-      <c r="B61" s="43" t="s">
-        <v>195</v>
-      </c>
-      <c r="C61" s="46" t="s">
+      <c r="B61" s="39" t="s">
+        <v>195</v>
+      </c>
+      <c r="C61" s="42" t="s">
         <v>14</v>
       </c>
-      <c r="D61" s="46" t="s">
+      <c r="D61" s="42" t="s">
         <v>15</v>
       </c>
-      <c r="E61" s="47" t="s">
+      <c r="E61" s="43" t="s">
         <v>16</v>
       </c>
-      <c r="F61" s="48" t="s">
+      <c r="F61" s="44" t="s">
         <v>17</v>
       </c>
-      <c r="G61" s="49" t="s">
+      <c r="G61" s="45" t="s">
         <v>18</v>
       </c>
-      <c r="H61" s="50" t="s">
+      <c r="H61" s="34" t="s">
         <v>59</v>
       </c>
-      <c r="I61" s="50" t="s">
+      <c r="I61" s="34" t="s">
         <v>15</v>
       </c>
-      <c r="J61" s="50" t="s">
+      <c r="J61" s="34" t="s">
         <v>20</v>
       </c>
-      <c r="K61" s="50" t="s">
+      <c r="K61" s="34" t="s">
         <v>60</v>
       </c>
-      <c r="L61" s="50" t="s">
+      <c r="L61" s="34" t="s">
         <v>15</v>
       </c>
-      <c r="M61" s="50" t="s">
+      <c r="M61" s="34" t="s">
         <v>20</v>
       </c>
-      <c r="N61" s="50" t="s">
+      <c r="N61" s="34" t="s">
         <v>61</v>
       </c>
-      <c r="O61" s="50" t="s">
+      <c r="O61" s="34" t="s">
         <v>15</v>
       </c>
-      <c r="P61" s="50" t="s">
+      <c r="P61" s="34" t="s">
         <v>20</v>
       </c>
-      <c r="Q61" s="50" t="s">
+      <c r="Q61" s="34" t="s">
         <v>62</v>
       </c>
-      <c r="R61" s="50" t="s">
+      <c r="R61" s="34" t="s">
         <v>15</v>
       </c>
-      <c r="S61" s="50" t="s">
+      <c r="S61" s="34" t="s">
         <v>20</v>
       </c>
-      <c r="T61" s="41" t="s">
+      <c r="T61" s="46" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="62" spans="1:20" ht="13" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A62" s="43" t="s">
-        <v>195</v>
-      </c>
-      <c r="B62" s="43" t="s">
-        <v>195</v>
-      </c>
-      <c r="C62" s="46" t="s">
-        <v>195</v>
-      </c>
-      <c r="D62" s="46" t="s">
-        <v>195</v>
-      </c>
-      <c r="E62" s="47" t="s">
-        <v>195</v>
-      </c>
-      <c r="F62" s="48" t="s">
-        <v>195</v>
-      </c>
-      <c r="G62" s="49" t="s">
-        <v>195</v>
-      </c>
-      <c r="H62" s="51" t="s">
+      <c r="A62" s="39" t="s">
+        <v>195</v>
+      </c>
+      <c r="B62" s="39" t="s">
+        <v>195</v>
+      </c>
+      <c r="C62" s="42" t="s">
+        <v>195</v>
+      </c>
+      <c r="D62" s="42" t="s">
+        <v>195</v>
+      </c>
+      <c r="E62" s="43" t="s">
+        <v>195</v>
+      </c>
+      <c r="F62" s="44" t="s">
+        <v>195</v>
+      </c>
+      <c r="G62" s="45" t="s">
+        <v>195</v>
+      </c>
+      <c r="H62" s="35" t="s">
         <v>63</v>
       </c>
-      <c r="I62" s="51" t="s">
-        <v>195</v>
-      </c>
-      <c r="J62" s="51" t="s">
-        <v>195</v>
-      </c>
-      <c r="K62" s="51" t="s">
+      <c r="I62" s="35" t="s">
+        <v>195</v>
+      </c>
+      <c r="J62" s="35" t="s">
+        <v>195</v>
+      </c>
+      <c r="K62" s="35" t="s">
         <v>64</v>
       </c>
-      <c r="L62" s="51" t="s">
-        <v>195</v>
-      </c>
-      <c r="M62" s="51" t="s">
-        <v>195</v>
-      </c>
-      <c r="N62" s="51" t="s">
+      <c r="L62" s="35" t="s">
+        <v>195</v>
+      </c>
+      <c r="M62" s="35" t="s">
+        <v>195</v>
+      </c>
+      <c r="N62" s="35" t="s">
         <v>65</v>
       </c>
-      <c r="O62" s="51" t="s">
-        <v>195</v>
-      </c>
-      <c r="P62" s="51" t="s">
-        <v>195</v>
-      </c>
-      <c r="Q62" s="51" t="s">
+      <c r="O62" s="35" t="s">
+        <v>195</v>
+      </c>
+      <c r="P62" s="35" t="s">
+        <v>195</v>
+      </c>
+      <c r="Q62" s="35" t="s">
         <v>50</v>
       </c>
-      <c r="R62" s="51" t="s">
-        <v>195</v>
-      </c>
-      <c r="S62" s="51" t="s">
-        <v>195</v>
-      </c>
-      <c r="T62" s="41" t="s">
+      <c r="R62" s="35" t="s">
+        <v>195</v>
+      </c>
+      <c r="S62" s="35" t="s">
+        <v>195</v>
+      </c>
+      <c r="T62" s="46" t="s">
         <v>195</v>
       </c>
     </row>
     <row r="63" spans="1:20" ht="22" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A63" s="43" t="s">
+      <c r="A63" s="39" t="s">
         <v>13</v>
       </c>
-      <c r="B63" s="43" t="s">
-        <v>195</v>
-      </c>
-      <c r="C63" s="46" t="s">
+      <c r="B63" s="39" t="s">
+        <v>195</v>
+      </c>
+      <c r="C63" s="42" t="s">
         <v>14</v>
       </c>
-      <c r="D63" s="46" t="s">
+      <c r="D63" s="42" t="s">
         <v>15</v>
       </c>
-      <c r="E63" s="47" t="s">
+      <c r="E63" s="43" t="s">
         <v>16</v>
       </c>
-      <c r="F63" s="48" t="s">
+      <c r="F63" s="44" t="s">
         <v>17</v>
       </c>
-      <c r="G63" s="49" t="s">
+      <c r="G63" s="45" t="s">
         <v>18</v>
       </c>
       <c r="H63" s="17" t="s">
@@ -5465,7 +5465,7 @@
       <c r="S63" s="19" t="s">
         <v>20</v>
       </c>
-      <c r="T63" s="41" t="s">
+      <c r="T63" s="46" t="s">
         <v>24</v>
       </c>
     </row>
@@ -5808,41 +5808,41 @@
       <c r="B70" s="20"/>
       <c r="C70" s="20"/>
       <c r="D70" s="20"/>
-      <c r="E70" s="44" t="s">
+      <c r="E70" s="40" t="s">
         <v>43</v>
       </c>
-      <c r="F70" s="44"/>
-      <c r="G70" s="45"/>
-      <c r="H70" s="52">
+      <c r="F70" s="40"/>
+      <c r="G70" s="41"/>
+      <c r="H70" s="36">
         <v>2783.5147247314453</v>
       </c>
-      <c r="I70" s="53"/>
-      <c r="J70" s="54"/>
-      <c r="K70" s="52">
+      <c r="I70" s="37"/>
+      <c r="J70" s="38"/>
+      <c r="K70" s="36">
         <v>2293</v>
       </c>
-      <c r="L70" s="53"/>
-      <c r="M70" s="54"/>
-      <c r="N70" s="52">
+      <c r="L70" s="37"/>
+      <c r="M70" s="38"/>
+      <c r="N70" s="36">
         <v>1529.7916666666665</v>
       </c>
-      <c r="O70" s="53"/>
-      <c r="P70" s="54"/>
-      <c r="Q70" s="52">
+      <c r="O70" s="37"/>
+      <c r="P70" s="38"/>
+      <c r="Q70" s="36">
         <v>387</v>
       </c>
-      <c r="R70" s="53"/>
-      <c r="S70" s="54"/>
+      <c r="R70" s="37"/>
+      <c r="S70" s="38"/>
     </row>
     <row r="71" spans="1:20" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A71" s="21" t="s">
         <v>44</v>
       </c>
-      <c r="D71" s="39">
+      <c r="D71" s="47">
         <v>543.82320238095235</v>
       </c>
-      <c r="E71" s="35"/>
-      <c r="F71" s="35"/>
+      <c r="E71" s="48"/>
+      <c r="F71" s="48"/>
       <c r="G71" s="21" t="s">
         <v>45</v>
       </c>
@@ -5975,149 +5975,149 @@
       </c>
     </row>
     <row r="74" spans="1:20" ht="13" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A74" s="43" t="s">
+      <c r="A74" s="39" t="s">
         <v>13</v>
       </c>
-      <c r="B74" s="43" t="s">
-        <v>195</v>
-      </c>
-      <c r="C74" s="46" t="s">
+      <c r="B74" s="39" t="s">
+        <v>195</v>
+      </c>
+      <c r="C74" s="42" t="s">
         <v>14</v>
       </c>
-      <c r="D74" s="46" t="s">
+      <c r="D74" s="42" t="s">
         <v>15</v>
       </c>
-      <c r="E74" s="47" t="s">
+      <c r="E74" s="43" t="s">
         <v>16</v>
       </c>
-      <c r="F74" s="48" t="s">
+      <c r="F74" s="44" t="s">
         <v>17</v>
       </c>
-      <c r="G74" s="49" t="s">
+      <c r="G74" s="45" t="s">
         <v>18</v>
       </c>
-      <c r="H74" s="50" t="s">
+      <c r="H74" s="34" t="s">
         <v>66</v>
       </c>
-      <c r="I74" s="50" t="s">
+      <c r="I74" s="34" t="s">
         <v>15</v>
       </c>
-      <c r="J74" s="50" t="s">
+      <c r="J74" s="34" t="s">
         <v>20</v>
       </c>
-      <c r="K74" s="50" t="s">
+      <c r="K74" s="34" t="s">
         <v>67</v>
       </c>
-      <c r="L74" s="50" t="s">
+      <c r="L74" s="34" t="s">
         <v>15</v>
       </c>
-      <c r="M74" s="50" t="s">
+      <c r="M74" s="34" t="s">
         <v>20</v>
       </c>
-      <c r="N74" s="50" t="s">
+      <c r="N74" s="34" t="s">
         <v>68</v>
       </c>
-      <c r="O74" s="50" t="s">
+      <c r="O74" s="34" t="s">
         <v>15</v>
       </c>
-      <c r="P74" s="50" t="s">
+      <c r="P74" s="34" t="s">
         <v>20</v>
       </c>
-      <c r="Q74" s="50" t="s">
+      <c r="Q74" s="34" t="s">
         <v>69</v>
       </c>
-      <c r="R74" s="50" t="s">
+      <c r="R74" s="34" t="s">
         <v>15</v>
       </c>
-      <c r="S74" s="50" t="s">
+      <c r="S74" s="34" t="s">
         <v>20</v>
       </c>
-      <c r="T74" s="41" t="s">
+      <c r="T74" s="46" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="75" spans="1:20" ht="13" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A75" s="43" t="s">
-        <v>195</v>
-      </c>
-      <c r="B75" s="43" t="s">
-        <v>195</v>
-      </c>
-      <c r="C75" s="46" t="s">
-        <v>195</v>
-      </c>
-      <c r="D75" s="46" t="s">
-        <v>195</v>
-      </c>
-      <c r="E75" s="47" t="s">
-        <v>195</v>
-      </c>
-      <c r="F75" s="48" t="s">
-        <v>195</v>
-      </c>
-      <c r="G75" s="49" t="s">
-        <v>195</v>
-      </c>
-      <c r="H75" s="51" t="s">
+      <c r="A75" s="39" t="s">
+        <v>195</v>
+      </c>
+      <c r="B75" s="39" t="s">
+        <v>195</v>
+      </c>
+      <c r="C75" s="42" t="s">
+        <v>195</v>
+      </c>
+      <c r="D75" s="42" t="s">
+        <v>195</v>
+      </c>
+      <c r="E75" s="43" t="s">
+        <v>195</v>
+      </c>
+      <c r="F75" s="44" t="s">
+        <v>195</v>
+      </c>
+      <c r="G75" s="45" t="s">
+        <v>195</v>
+      </c>
+      <c r="H75" s="35" t="s">
         <v>50</v>
       </c>
-      <c r="I75" s="51" t="s">
-        <v>195</v>
-      </c>
-      <c r="J75" s="51" t="s">
-        <v>195</v>
-      </c>
-      <c r="K75" s="51" t="s">
+      <c r="I75" s="35" t="s">
+        <v>195</v>
+      </c>
+      <c r="J75" s="35" t="s">
+        <v>195</v>
+      </c>
+      <c r="K75" s="35" t="s">
         <v>63</v>
       </c>
-      <c r="L75" s="51" t="s">
-        <v>195</v>
-      </c>
-      <c r="M75" s="51" t="s">
-        <v>195</v>
-      </c>
-      <c r="N75" s="51" t="s">
+      <c r="L75" s="35" t="s">
+        <v>195</v>
+      </c>
+      <c r="M75" s="35" t="s">
+        <v>195</v>
+      </c>
+      <c r="N75" s="35" t="s">
         <v>28</v>
       </c>
-      <c r="O75" s="51" t="s">
-        <v>195</v>
-      </c>
-      <c r="P75" s="51" t="s">
-        <v>195</v>
-      </c>
-      <c r="Q75" s="51" t="s">
+      <c r="O75" s="35" t="s">
+        <v>195</v>
+      </c>
+      <c r="P75" s="35" t="s">
+        <v>195</v>
+      </c>
+      <c r="Q75" s="35" t="s">
         <v>65</v>
       </c>
-      <c r="R75" s="51" t="s">
-        <v>195</v>
-      </c>
-      <c r="S75" s="51" t="s">
-        <v>195</v>
-      </c>
-      <c r="T75" s="41" t="s">
+      <c r="R75" s="35" t="s">
+        <v>195</v>
+      </c>
+      <c r="S75" s="35" t="s">
+        <v>195</v>
+      </c>
+      <c r="T75" s="46" t="s">
         <v>195</v>
       </c>
     </row>
     <row r="76" spans="1:20" ht="22" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A76" s="43" t="s">
+      <c r="A76" s="39" t="s">
         <v>13</v>
       </c>
-      <c r="B76" s="43" t="s">
-        <v>195</v>
-      </c>
-      <c r="C76" s="46" t="s">
+      <c r="B76" s="39" t="s">
+        <v>195</v>
+      </c>
+      <c r="C76" s="42" t="s">
         <v>14</v>
       </c>
-      <c r="D76" s="46" t="s">
+      <c r="D76" s="42" t="s">
         <v>15</v>
       </c>
-      <c r="E76" s="47" t="s">
+      <c r="E76" s="43" t="s">
         <v>16</v>
       </c>
-      <c r="F76" s="48" t="s">
+      <c r="F76" s="44" t="s">
         <v>17</v>
       </c>
-      <c r="G76" s="49" t="s">
+      <c r="G76" s="45" t="s">
         <v>18</v>
       </c>
       <c r="H76" s="17" t="s">
@@ -6156,7 +6156,7 @@
       <c r="S76" s="19" t="s">
         <v>20</v>
       </c>
-      <c r="T76" s="41" t="s">
+      <c r="T76" s="46" t="s">
         <v>24</v>
       </c>
     </row>
@@ -6493,41 +6493,41 @@
       <c r="B83" s="20"/>
       <c r="C83" s="20"/>
       <c r="D83" s="20"/>
-      <c r="E83" s="44" t="s">
+      <c r="E83" s="40" t="s">
         <v>43</v>
       </c>
-      <c r="F83" s="44"/>
-      <c r="G83" s="45"/>
-      <c r="H83" s="52">
+      <c r="F83" s="40"/>
+      <c r="G83" s="41"/>
+      <c r="H83" s="36">
         <v>103</v>
       </c>
-      <c r="I83" s="53"/>
-      <c r="J83" s="54"/>
-      <c r="K83" s="52">
+      <c r="I83" s="37"/>
+      <c r="J83" s="38"/>
+      <c r="K83" s="36">
         <v>2208.5</v>
       </c>
-      <c r="L83" s="53"/>
-      <c r="M83" s="54"/>
-      <c r="N83" s="52">
+      <c r="L83" s="37"/>
+      <c r="M83" s="38"/>
+      <c r="N83" s="36">
         <v>1168.5</v>
       </c>
-      <c r="O83" s="53"/>
-      <c r="P83" s="54"/>
-      <c r="Q83" s="52">
+      <c r="O83" s="37"/>
+      <c r="P83" s="38"/>
+      <c r="Q83" s="36">
         <v>2379.723401248455</v>
       </c>
-      <c r="R83" s="53"/>
-      <c r="S83" s="54"/>
+      <c r="R83" s="37"/>
+      <c r="S83" s="38"/>
     </row>
     <row r="84" spans="1:20" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A84" s="21" t="s">
         <v>44</v>
       </c>
-      <c r="D84" s="39">
+      <c r="D84" s="47">
         <v>543.82320238095235</v>
       </c>
-      <c r="E84" s="35"/>
-      <c r="F84" s="35"/>
+      <c r="E84" s="48"/>
+      <c r="F84" s="48"/>
       <c r="G84" s="21" t="s">
         <v>45</v>
       </c>
@@ -6846,149 +6846,149 @@
       </c>
     </row>
     <row r="90" spans="1:20" ht="13" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A90" s="43" t="s">
+      <c r="A90" s="39" t="s">
         <v>13</v>
       </c>
-      <c r="B90" s="43" t="s">
-        <v>195</v>
-      </c>
-      <c r="C90" s="46" t="s">
+      <c r="B90" s="39" t="s">
+        <v>195</v>
+      </c>
+      <c r="C90" s="42" t="s">
         <v>14</v>
       </c>
-      <c r="D90" s="46" t="s">
+      <c r="D90" s="42" t="s">
         <v>15</v>
       </c>
-      <c r="E90" s="47" t="s">
+      <c r="E90" s="43" t="s">
         <v>16</v>
       </c>
-      <c r="F90" s="48" t="s">
+      <c r="F90" s="44" t="s">
         <v>17</v>
       </c>
-      <c r="G90" s="49" t="s">
+      <c r="G90" s="45" t="s">
         <v>18</v>
       </c>
-      <c r="H90" s="50" t="s">
+      <c r="H90" s="34" t="s">
         <v>70</v>
       </c>
-      <c r="I90" s="50" t="s">
+      <c r="I90" s="34" t="s">
         <v>15</v>
       </c>
-      <c r="J90" s="50" t="s">
+      <c r="J90" s="34" t="s">
         <v>20</v>
       </c>
-      <c r="K90" s="50" t="s">
+      <c r="K90" s="34" t="s">
         <v>71</v>
       </c>
-      <c r="L90" s="50" t="s">
+      <c r="L90" s="34" t="s">
         <v>15</v>
       </c>
-      <c r="M90" s="50" t="s">
+      <c r="M90" s="34" t="s">
         <v>20</v>
       </c>
-      <c r="N90" s="50" t="s">
+      <c r="N90" s="34" t="s">
         <v>72</v>
       </c>
-      <c r="O90" s="50" t="s">
+      <c r="O90" s="34" t="s">
         <v>15</v>
       </c>
-      <c r="P90" s="50" t="s">
+      <c r="P90" s="34" t="s">
         <v>20</v>
       </c>
-      <c r="Q90" s="50" t="s">
+      <c r="Q90" s="34" t="s">
         <v>73</v>
       </c>
-      <c r="R90" s="50" t="s">
+      <c r="R90" s="34" t="s">
         <v>15</v>
       </c>
-      <c r="S90" s="50" t="s">
+      <c r="S90" s="34" t="s">
         <v>20</v>
       </c>
-      <c r="T90" s="41" t="s">
+      <c r="T90" s="46" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="91" spans="1:20" ht="13" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A91" s="43" t="s">
-        <v>195</v>
-      </c>
-      <c r="B91" s="43" t="s">
-        <v>195</v>
-      </c>
-      <c r="C91" s="46" t="s">
-        <v>195</v>
-      </c>
-      <c r="D91" s="46" t="s">
-        <v>195</v>
-      </c>
-      <c r="E91" s="47" t="s">
-        <v>195</v>
-      </c>
-      <c r="F91" s="48" t="s">
-        <v>195</v>
-      </c>
-      <c r="G91" s="49" t="s">
-        <v>195</v>
-      </c>
-      <c r="H91" s="51" t="s">
+      <c r="A91" s="39" t="s">
+        <v>195</v>
+      </c>
+      <c r="B91" s="39" t="s">
+        <v>195</v>
+      </c>
+      <c r="C91" s="42" t="s">
+        <v>195</v>
+      </c>
+      <c r="D91" s="42" t="s">
+        <v>195</v>
+      </c>
+      <c r="E91" s="43" t="s">
+        <v>195</v>
+      </c>
+      <c r="F91" s="44" t="s">
+        <v>195</v>
+      </c>
+      <c r="G91" s="45" t="s">
+        <v>195</v>
+      </c>
+      <c r="H91" s="35" t="s">
         <v>28</v>
       </c>
-      <c r="I91" s="51" t="s">
-        <v>195</v>
-      </c>
-      <c r="J91" s="51" t="s">
-        <v>195</v>
-      </c>
-      <c r="K91" s="51" t="s">
+      <c r="I91" s="35" t="s">
+        <v>195</v>
+      </c>
+      <c r="J91" s="35" t="s">
+        <v>195</v>
+      </c>
+      <c r="K91" s="35" t="s">
         <v>25</v>
       </c>
-      <c r="L91" s="51" t="s">
-        <v>195</v>
-      </c>
-      <c r="M91" s="51" t="s">
-        <v>195</v>
-      </c>
-      <c r="N91" s="51" t="s">
+      <c r="L91" s="35" t="s">
+        <v>195</v>
+      </c>
+      <c r="M91" s="35" t="s">
+        <v>195</v>
+      </c>
+      <c r="N91" s="35" t="s">
         <v>74</v>
       </c>
-      <c r="O91" s="51" t="s">
-        <v>195</v>
-      </c>
-      <c r="P91" s="51" t="s">
-        <v>195</v>
-      </c>
-      <c r="Q91" s="51" t="s">
+      <c r="O91" s="35" t="s">
+        <v>195</v>
+      </c>
+      <c r="P91" s="35" t="s">
+        <v>195</v>
+      </c>
+      <c r="Q91" s="35" t="s">
         <v>64</v>
       </c>
-      <c r="R91" s="51" t="s">
-        <v>195</v>
-      </c>
-      <c r="S91" s="51" t="s">
-        <v>195</v>
-      </c>
-      <c r="T91" s="41" t="s">
+      <c r="R91" s="35" t="s">
+        <v>195</v>
+      </c>
+      <c r="S91" s="35" t="s">
+        <v>195</v>
+      </c>
+      <c r="T91" s="46" t="s">
         <v>195</v>
       </c>
     </row>
     <row r="92" spans="1:20" ht="22" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A92" s="43" t="s">
+      <c r="A92" s="39" t="s">
         <v>13</v>
       </c>
-      <c r="B92" s="43" t="s">
-        <v>195</v>
-      </c>
-      <c r="C92" s="46" t="s">
+      <c r="B92" s="39" t="s">
+        <v>195</v>
+      </c>
+      <c r="C92" s="42" t="s">
         <v>14</v>
       </c>
-      <c r="D92" s="46" t="s">
+      <c r="D92" s="42" t="s">
         <v>15</v>
       </c>
-      <c r="E92" s="47" t="s">
+      <c r="E92" s="43" t="s">
         <v>16</v>
       </c>
-      <c r="F92" s="48" t="s">
+      <c r="F92" s="44" t="s">
         <v>17</v>
       </c>
-      <c r="G92" s="49" t="s">
+      <c r="G92" s="45" t="s">
         <v>18</v>
       </c>
       <c r="H92" s="17" t="s">
@@ -7027,7 +7027,7 @@
       <c r="S92" s="19" t="s">
         <v>20</v>
       </c>
-      <c r="T92" s="41" t="s">
+      <c r="T92" s="46" t="s">
         <v>24</v>
       </c>
     </row>
@@ -7390,41 +7390,41 @@
       <c r="B99" s="20"/>
       <c r="C99" s="20"/>
       <c r="D99" s="20"/>
-      <c r="E99" s="44" t="s">
+      <c r="E99" s="40" t="s">
         <v>43</v>
       </c>
-      <c r="F99" s="44"/>
-      <c r="G99" s="45"/>
-      <c r="H99" s="52">
+      <c r="F99" s="40"/>
+      <c r="G99" s="41"/>
+      <c r="H99" s="36">
         <v>1223.5</v>
       </c>
-      <c r="I99" s="53"/>
-      <c r="J99" s="54"/>
-      <c r="K99" s="52">
+      <c r="I99" s="37"/>
+      <c r="J99" s="38"/>
+      <c r="K99" s="36">
         <v>5909.1111111111113</v>
       </c>
-      <c r="L99" s="53"/>
-      <c r="M99" s="54"/>
-      <c r="N99" s="52">
+      <c r="L99" s="37"/>
+      <c r="M99" s="38"/>
+      <c r="N99" s="36">
         <v>4410.25</v>
       </c>
-      <c r="O99" s="53"/>
-      <c r="P99" s="54"/>
-      <c r="Q99" s="52">
+      <c r="O99" s="37"/>
+      <c r="P99" s="38"/>
+      <c r="Q99" s="36">
         <v>2174.908447265625</v>
       </c>
-      <c r="R99" s="53"/>
-      <c r="S99" s="54"/>
+      <c r="R99" s="37"/>
+      <c r="S99" s="38"/>
     </row>
     <row r="100" spans="1:20" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A100" s="21" t="s">
         <v>44</v>
       </c>
-      <c r="D100" s="39">
+      <c r="D100" s="47">
         <v>543.82320238095235</v>
       </c>
-      <c r="E100" s="35"/>
-      <c r="F100" s="35"/>
+      <c r="E100" s="48"/>
+      <c r="F100" s="48"/>
       <c r="G100" s="21" t="s">
         <v>45</v>
       </c>
@@ -7557,113 +7557,113 @@
       </c>
     </row>
     <row r="103" spans="1:20" ht="13" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A103" s="43" t="s">
+      <c r="A103" s="39" t="s">
         <v>13</v>
       </c>
-      <c r="B103" s="43" t="s">
-        <v>195</v>
-      </c>
-      <c r="C103" s="46" t="s">
+      <c r="B103" s="39" t="s">
+        <v>195</v>
+      </c>
+      <c r="C103" s="42" t="s">
         <v>14</v>
       </c>
-      <c r="D103" s="46" t="s">
+      <c r="D103" s="42" t="s">
         <v>15</v>
       </c>
-      <c r="E103" s="47" t="s">
+      <c r="E103" s="43" t="s">
         <v>16</v>
       </c>
-      <c r="F103" s="48" t="s">
+      <c r="F103" s="44" t="s">
         <v>17</v>
       </c>
-      <c r="G103" s="49" t="s">
+      <c r="G103" s="45" t="s">
         <v>18</v>
       </c>
-      <c r="H103" s="50" t="s">
+      <c r="H103" s="34" t="s">
         <v>75</v>
       </c>
-      <c r="I103" s="50" t="s">
+      <c r="I103" s="34" t="s">
         <v>15</v>
       </c>
-      <c r="J103" s="50" t="s">
+      <c r="J103" s="34" t="s">
         <v>20</v>
       </c>
-      <c r="K103" s="50" t="s">
+      <c r="K103" s="34" t="s">
         <v>76</v>
       </c>
-      <c r="L103" s="50" t="s">
+      <c r="L103" s="34" t="s">
         <v>15</v>
       </c>
-      <c r="M103" s="50" t="s">
+      <c r="M103" s="34" t="s">
         <v>20</v>
       </c>
-      <c r="N103" s="41" t="s">
+      <c r="N103" s="46" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="104" spans="1:20" ht="13" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A104" s="43" t="s">
-        <v>195</v>
-      </c>
-      <c r="B104" s="43" t="s">
-        <v>195</v>
-      </c>
-      <c r="C104" s="46" t="s">
-        <v>195</v>
-      </c>
-      <c r="D104" s="46" t="s">
-        <v>195</v>
-      </c>
-      <c r="E104" s="47" t="s">
-        <v>195</v>
-      </c>
-      <c r="F104" s="48" t="s">
-        <v>195</v>
-      </c>
-      <c r="G104" s="49" t="s">
-        <v>195</v>
-      </c>
-      <c r="H104" s="51" t="s">
+      <c r="A104" s="39" t="s">
+        <v>195</v>
+      </c>
+      <c r="B104" s="39" t="s">
+        <v>195</v>
+      </c>
+      <c r="C104" s="42" t="s">
+        <v>195</v>
+      </c>
+      <c r="D104" s="42" t="s">
+        <v>195</v>
+      </c>
+      <c r="E104" s="43" t="s">
+        <v>195</v>
+      </c>
+      <c r="F104" s="44" t="s">
+        <v>195</v>
+      </c>
+      <c r="G104" s="45" t="s">
+        <v>195</v>
+      </c>
+      <c r="H104" s="35" t="s">
         <v>77</v>
       </c>
-      <c r="I104" s="51" t="s">
-        <v>195</v>
-      </c>
-      <c r="J104" s="51" t="s">
-        <v>195</v>
-      </c>
-      <c r="K104" s="51" t="s">
+      <c r="I104" s="35" t="s">
+        <v>195</v>
+      </c>
+      <c r="J104" s="35" t="s">
+        <v>195</v>
+      </c>
+      <c r="K104" s="35" t="s">
         <v>65</v>
       </c>
-      <c r="L104" s="51" t="s">
-        <v>195</v>
-      </c>
-      <c r="M104" s="51" t="s">
-        <v>195</v>
-      </c>
-      <c r="N104" s="42">
+      <c r="L104" s="35" t="s">
+        <v>195</v>
+      </c>
+      <c r="M104" s="35" t="s">
+        <v>195</v>
+      </c>
+      <c r="N104" s="50">
         <v>0</v>
       </c>
     </row>
     <row r="105" spans="1:20" ht="22" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A105" s="43" t="s">
+      <c r="A105" s="39" t="s">
         <v>13</v>
       </c>
-      <c r="B105" s="43" t="s">
-        <v>195</v>
-      </c>
-      <c r="C105" s="46" t="s">
+      <c r="B105" s="39" t="s">
+        <v>195</v>
+      </c>
+      <c r="C105" s="42" t="s">
         <v>14</v>
       </c>
-      <c r="D105" s="46" t="s">
+      <c r="D105" s="42" t="s">
         <v>15</v>
       </c>
-      <c r="E105" s="47" t="s">
+      <c r="E105" s="43" t="s">
         <v>16</v>
       </c>
-      <c r="F105" s="48" t="s">
+      <c r="F105" s="44" t="s">
         <v>17</v>
       </c>
-      <c r="G105" s="49" t="s">
+      <c r="G105" s="45" t="s">
         <v>18</v>
       </c>
       <c r="H105" s="17" t="s">
@@ -7684,7 +7684,7 @@
       <c r="M105" s="19" t="s">
         <v>20</v>
       </c>
-      <c r="N105" s="42">
+      <c r="N105" s="50">
         <v>0</v>
       </c>
     </row>
@@ -7947,31 +7947,31 @@
       <c r="B112" s="20"/>
       <c r="C112" s="20"/>
       <c r="D112" s="20"/>
-      <c r="E112" s="44" t="s">
+      <c r="E112" s="40" t="s">
         <v>43</v>
       </c>
-      <c r="F112" s="44"/>
-      <c r="G112" s="45"/>
-      <c r="H112" s="52">
+      <c r="F112" s="40"/>
+      <c r="G112" s="41"/>
+      <c r="H112" s="36">
         <v>4614.1000000000004</v>
       </c>
-      <c r="I112" s="53"/>
-      <c r="J112" s="54"/>
-      <c r="K112" s="52">
+      <c r="I112" s="37"/>
+      <c r="J112" s="38"/>
+      <c r="K112" s="36">
         <v>1555.2778244018546</v>
       </c>
-      <c r="L112" s="53"/>
-      <c r="M112" s="54"/>
+      <c r="L112" s="37"/>
+      <c r="M112" s="38"/>
     </row>
     <row r="113" spans="1:20" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A113" s="21" t="s">
         <v>44</v>
       </c>
-      <c r="D113" s="39">
+      <c r="D113" s="47">
         <v>543.82320238095235</v>
       </c>
-      <c r="E113" s="35"/>
-      <c r="F113" s="35"/>
+      <c r="E113" s="48"/>
+      <c r="F113" s="48"/>
       <c r="G113" s="21" t="s">
         <v>45</v>
       </c>
@@ -8166,88 +8166,88 @@
       </c>
     </row>
     <row r="117" spans="1:20" ht="16" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A117" s="40" t="s">
+      <c r="A117" s="49" t="s">
         <v>78</v>
       </c>
-      <c r="B117" s="35"/>
-      <c r="C117" s="35"/>
-      <c r="D117" s="35"/>
-      <c r="E117" s="35"/>
-      <c r="F117" s="35"/>
-      <c r="G117" s="35"/>
-      <c r="H117" s="35"/>
-      <c r="I117" s="35"/>
-      <c r="J117" s="35"/>
-      <c r="K117" s="35"/>
-      <c r="L117" s="35"/>
-      <c r="M117" s="35"/>
-      <c r="N117" s="35"/>
-      <c r="O117" s="35"/>
-      <c r="P117" s="35"/>
-      <c r="Q117" s="35"/>
-      <c r="R117" s="35"/>
-      <c r="S117" s="35"/>
-      <c r="T117" s="35"/>
+      <c r="B117" s="48"/>
+      <c r="C117" s="48"/>
+      <c r="D117" s="48"/>
+      <c r="E117" s="48"/>
+      <c r="F117" s="48"/>
+      <c r="G117" s="48"/>
+      <c r="H117" s="48"/>
+      <c r="I117" s="48"/>
+      <c r="J117" s="48"/>
+      <c r="K117" s="48"/>
+      <c r="L117" s="48"/>
+      <c r="M117" s="48"/>
+      <c r="N117" s="48"/>
+      <c r="O117" s="48"/>
+      <c r="P117" s="48"/>
+      <c r="Q117" s="48"/>
+      <c r="R117" s="48"/>
+      <c r="S117" s="48"/>
+      <c r="T117" s="48"/>
     </row>
     <row r="118" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A118" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="B118" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="C118" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="D118" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="E118" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="F118" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="G118" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="H118" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="I118" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="J118" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="K118" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="L118" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="M118" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="N118" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="O118" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="P118" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="Q118" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="R118" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="S118" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="T118" s="35" t="s">
+      <c r="A118" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="B118" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="C118" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="D118" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="E118" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="F118" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="G118" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="H118" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="I118" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="J118" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="K118" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="L118" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="M118" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="N118" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="O118" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="P118" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="Q118" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="R118" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="S118" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="T118" s="48" t="s">
         <v>195</v>
       </c>
     </row>
@@ -8314,212 +8314,212 @@
       </c>
     </row>
     <row r="120" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A120" s="40" t="s">
+      <c r="A120" s="49" t="s">
         <v>79</v>
       </c>
-      <c r="B120" s="35"/>
-      <c r="C120" s="35"/>
-      <c r="D120" s="35"/>
-      <c r="E120" s="35"/>
-      <c r="F120" s="35"/>
-      <c r="G120" s="35"/>
-      <c r="H120" s="35"/>
-      <c r="I120" s="35"/>
-      <c r="J120" s="35"/>
-      <c r="K120" s="35"/>
-      <c r="L120" s="35"/>
-      <c r="M120" s="35"/>
-      <c r="N120" s="35"/>
-      <c r="O120" s="35"/>
-      <c r="P120" s="35"/>
-      <c r="Q120" s="35"/>
-      <c r="R120" s="35"/>
-      <c r="S120" s="35"/>
-      <c r="T120" s="35"/>
+      <c r="B120" s="48"/>
+      <c r="C120" s="48"/>
+      <c r="D120" s="48"/>
+      <c r="E120" s="48"/>
+      <c r="F120" s="48"/>
+      <c r="G120" s="48"/>
+      <c r="H120" s="48"/>
+      <c r="I120" s="48"/>
+      <c r="J120" s="48"/>
+      <c r="K120" s="48"/>
+      <c r="L120" s="48"/>
+      <c r="M120" s="48"/>
+      <c r="N120" s="48"/>
+      <c r="O120" s="48"/>
+      <c r="P120" s="48"/>
+      <c r="Q120" s="48"/>
+      <c r="R120" s="48"/>
+      <c r="S120" s="48"/>
+      <c r="T120" s="48"/>
     </row>
     <row r="121" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A121" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="B121" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="C121" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="D121" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="E121" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="F121" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="G121" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="H121" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="I121" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="J121" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="K121" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="L121" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="M121" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="N121" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="O121" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="P121" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="Q121" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="R121" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="S121" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="T121" s="35" t="s">
+      <c r="A121" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="B121" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="C121" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="D121" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="E121" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="F121" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="G121" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="H121" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="I121" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="J121" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="K121" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="L121" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="M121" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="N121" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="O121" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="P121" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="Q121" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="R121" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="S121" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="T121" s="48" t="s">
         <v>195</v>
       </c>
     </row>
     <row r="122" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A122" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="B122" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="C122" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="D122" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="E122" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="F122" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="G122" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="H122" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="I122" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="J122" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="K122" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="L122" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="M122" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="N122" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="O122" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="P122" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="Q122" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="R122" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="S122" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="T122" s="35" t="s">
+      <c r="A122" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="B122" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="C122" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="D122" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="E122" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="F122" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="G122" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="H122" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="I122" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="J122" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="K122" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="L122" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="M122" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="N122" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="O122" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="P122" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="Q122" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="R122" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="S122" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="T122" s="48" t="s">
         <v>195</v>
       </c>
     </row>
     <row r="123" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A123" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="B123" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="C123" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="D123" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="E123" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="F123" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="G123" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="H123" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="I123" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="J123" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="K123" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="L123" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="M123" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="N123" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="O123" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="P123" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="Q123" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="R123" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="S123" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="T123" s="35" t="s">
+      <c r="A123" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="B123" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="C123" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="D123" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="E123" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="F123" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="G123" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="H123" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="I123" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="J123" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="K123" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="L123" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="M123" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="N123" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="O123" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="P123" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="Q123" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="R123" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="S123" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="T123" s="48" t="s">
         <v>195</v>
       </c>
     </row>
@@ -8586,274 +8586,274 @@
       </c>
     </row>
     <row r="125" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A125" s="40" t="s">
+      <c r="A125" s="49" t="s">
         <v>80</v>
       </c>
-      <c r="B125" s="35"/>
-      <c r="C125" s="35"/>
-      <c r="D125" s="35"/>
-      <c r="E125" s="35"/>
-      <c r="F125" s="35"/>
-      <c r="G125" s="35"/>
-      <c r="H125" s="35"/>
-      <c r="I125" s="35"/>
-      <c r="J125" s="35"/>
-      <c r="K125" s="35"/>
-      <c r="L125" s="35"/>
-      <c r="M125" s="35"/>
-      <c r="N125" s="35"/>
-      <c r="O125" s="35"/>
-      <c r="P125" s="35"/>
-      <c r="Q125" s="35"/>
-      <c r="R125" s="35"/>
-      <c r="S125" s="35"/>
-      <c r="T125" s="35"/>
+      <c r="B125" s="48"/>
+      <c r="C125" s="48"/>
+      <c r="D125" s="48"/>
+      <c r="E125" s="48"/>
+      <c r="F125" s="48"/>
+      <c r="G125" s="48"/>
+      <c r="H125" s="48"/>
+      <c r="I125" s="48"/>
+      <c r="J125" s="48"/>
+      <c r="K125" s="48"/>
+      <c r="L125" s="48"/>
+      <c r="M125" s="48"/>
+      <c r="N125" s="48"/>
+      <c r="O125" s="48"/>
+      <c r="P125" s="48"/>
+      <c r="Q125" s="48"/>
+      <c r="R125" s="48"/>
+      <c r="S125" s="48"/>
+      <c r="T125" s="48"/>
     </row>
     <row r="126" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A126" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="B126" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="C126" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="D126" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="E126" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="F126" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="G126" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="H126" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="I126" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="J126" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="K126" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="L126" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="M126" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="N126" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="O126" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="P126" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="Q126" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="R126" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="S126" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="T126" s="35" t="s">
+      <c r="A126" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="B126" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="C126" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="D126" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="E126" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="F126" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="G126" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="H126" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="I126" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="J126" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="K126" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="L126" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="M126" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="N126" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="O126" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="P126" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="Q126" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="R126" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="S126" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="T126" s="48" t="s">
         <v>195</v>
       </c>
     </row>
     <row r="127" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A127" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="B127" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="C127" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="D127" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="E127" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="F127" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="G127" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="H127" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="I127" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="J127" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="K127" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="L127" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="M127" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="N127" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="O127" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="P127" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="Q127" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="R127" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="S127" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="T127" s="35" t="s">
+      <c r="A127" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="B127" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="C127" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="D127" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="E127" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="F127" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="G127" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="H127" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="I127" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="J127" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="K127" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="L127" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="M127" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="N127" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="O127" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="P127" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="Q127" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="R127" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="S127" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="T127" s="48" t="s">
         <v>195</v>
       </c>
     </row>
     <row r="128" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A128" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="B128" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="C128" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="D128" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="E128" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="F128" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="G128" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="H128" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="I128" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="J128" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="K128" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="L128" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="M128" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="N128" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="O128" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="P128" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="Q128" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="R128" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="S128" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="T128" s="35" t="s">
+      <c r="A128" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="B128" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="C128" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="D128" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="E128" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="F128" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="G128" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="H128" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="I128" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="J128" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="K128" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="L128" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="M128" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="N128" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="O128" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="P128" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="Q128" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="R128" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="S128" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="T128" s="48" t="s">
         <v>195</v>
       </c>
     </row>
     <row r="129" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A129" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="B129" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="C129" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="D129" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="E129" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="F129" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="G129" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="H129" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="I129" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="J129" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="K129" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="L129" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="M129" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="N129" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="O129" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="P129" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="Q129" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="R129" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="S129" s="35" t="s">
-        <v>195</v>
-      </c>
-      <c r="T129" s="35" t="s">
+      <c r="A129" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="B129" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="C129" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="D129" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="E129" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="F129" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="G129" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="H129" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="I129" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="J129" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="K129" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="L129" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="M129" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="N129" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="O129" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="P129" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="Q129" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="R129" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="S129" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="T129" s="48" t="s">
         <v>195</v>
       </c>
     </row>
@@ -8921,125 +8921,30 @@
     </row>
   </sheetData>
   <mergeCells count="167">
-    <mergeCell ref="K103:M103"/>
-    <mergeCell ref="K104:M104"/>
-    <mergeCell ref="K112:M112"/>
-    <mergeCell ref="A103:B105"/>
-    <mergeCell ref="E112:G112"/>
-    <mergeCell ref="C103:C105"/>
-    <mergeCell ref="D103:D105"/>
-    <mergeCell ref="E103:E105"/>
-    <mergeCell ref="F103:F105"/>
-    <mergeCell ref="G103:G105"/>
-    <mergeCell ref="H103:J103"/>
-    <mergeCell ref="H104:J104"/>
-    <mergeCell ref="H112:J112"/>
-    <mergeCell ref="A90:B92"/>
-    <mergeCell ref="E99:G99"/>
-    <mergeCell ref="C90:C92"/>
-    <mergeCell ref="D90:D92"/>
-    <mergeCell ref="E90:E92"/>
-    <mergeCell ref="F90:F92"/>
-    <mergeCell ref="G90:G92"/>
-    <mergeCell ref="T90:T92"/>
-    <mergeCell ref="H90:J90"/>
-    <mergeCell ref="H91:J91"/>
-    <mergeCell ref="H99:J99"/>
-    <mergeCell ref="K90:M90"/>
-    <mergeCell ref="K91:M91"/>
-    <mergeCell ref="K99:M99"/>
-    <mergeCell ref="N90:P90"/>
-    <mergeCell ref="N91:P91"/>
-    <mergeCell ref="N99:P99"/>
-    <mergeCell ref="Q90:S90"/>
-    <mergeCell ref="Q91:S91"/>
-    <mergeCell ref="Q99:S99"/>
-    <mergeCell ref="A74:B76"/>
-    <mergeCell ref="E83:G83"/>
-    <mergeCell ref="C74:C76"/>
-    <mergeCell ref="D74:D76"/>
-    <mergeCell ref="E74:E76"/>
-    <mergeCell ref="F74:F76"/>
-    <mergeCell ref="G74:G76"/>
-    <mergeCell ref="T74:T76"/>
-    <mergeCell ref="H74:J74"/>
-    <mergeCell ref="H75:J75"/>
-    <mergeCell ref="H83:J83"/>
-    <mergeCell ref="K74:M74"/>
-    <mergeCell ref="K75:M75"/>
-    <mergeCell ref="K83:M83"/>
-    <mergeCell ref="N74:P74"/>
-    <mergeCell ref="N75:P75"/>
-    <mergeCell ref="N83:P83"/>
-    <mergeCell ref="Q74:S74"/>
-    <mergeCell ref="Q75:S75"/>
-    <mergeCell ref="Q83:S83"/>
-    <mergeCell ref="A61:B63"/>
-    <mergeCell ref="E70:G70"/>
-    <mergeCell ref="C61:C63"/>
-    <mergeCell ref="D61:D63"/>
-    <mergeCell ref="E61:E63"/>
-    <mergeCell ref="F61:F63"/>
-    <mergeCell ref="G61:G63"/>
-    <mergeCell ref="T61:T63"/>
-    <mergeCell ref="H61:J61"/>
-    <mergeCell ref="H62:J62"/>
-    <mergeCell ref="H70:J70"/>
-    <mergeCell ref="K61:M61"/>
-    <mergeCell ref="K62:M62"/>
-    <mergeCell ref="K70:M70"/>
-    <mergeCell ref="N61:P61"/>
-    <mergeCell ref="N62:P62"/>
-    <mergeCell ref="N70:P70"/>
-    <mergeCell ref="Q61:S61"/>
-    <mergeCell ref="Q62:S62"/>
-    <mergeCell ref="Q70:S70"/>
-    <mergeCell ref="A48:B50"/>
-    <mergeCell ref="E57:G57"/>
-    <mergeCell ref="C48:C50"/>
-    <mergeCell ref="D48:D50"/>
-    <mergeCell ref="E48:E50"/>
-    <mergeCell ref="F48:F50"/>
-    <mergeCell ref="G48:G50"/>
-    <mergeCell ref="T48:T50"/>
-    <mergeCell ref="H48:J48"/>
-    <mergeCell ref="H49:J49"/>
-    <mergeCell ref="H57:J57"/>
-    <mergeCell ref="K48:M48"/>
-    <mergeCell ref="K49:M49"/>
-    <mergeCell ref="K57:M57"/>
-    <mergeCell ref="N48:P48"/>
-    <mergeCell ref="N49:P49"/>
-    <mergeCell ref="N57:P57"/>
-    <mergeCell ref="Q48:S48"/>
-    <mergeCell ref="Q49:S49"/>
-    <mergeCell ref="Q57:S57"/>
-    <mergeCell ref="T32:T34"/>
-    <mergeCell ref="H32:J32"/>
-    <mergeCell ref="H33:J33"/>
-    <mergeCell ref="H41:J41"/>
-    <mergeCell ref="K32:M32"/>
-    <mergeCell ref="K33:M33"/>
-    <mergeCell ref="K41:M41"/>
-    <mergeCell ref="N32:P32"/>
-    <mergeCell ref="N33:P33"/>
-    <mergeCell ref="N41:P41"/>
-    <mergeCell ref="Q32:S32"/>
-    <mergeCell ref="Q33:S33"/>
-    <mergeCell ref="Q41:S41"/>
-    <mergeCell ref="N19:P19"/>
-    <mergeCell ref="N20:P20"/>
-    <mergeCell ref="N28:P28"/>
-    <mergeCell ref="Q19:S19"/>
-    <mergeCell ref="Q20:S20"/>
-    <mergeCell ref="Q28:S28"/>
-    <mergeCell ref="A32:B34"/>
-    <mergeCell ref="E41:G41"/>
-    <mergeCell ref="C32:C34"/>
-    <mergeCell ref="D32:D34"/>
-    <mergeCell ref="E32:E34"/>
-    <mergeCell ref="F32:F34"/>
-    <mergeCell ref="G32:G34"/>
+    <mergeCell ref="A2:T2"/>
+    <mergeCell ref="A3:T3"/>
+    <mergeCell ref="D16:F16"/>
+    <mergeCell ref="D29:F29"/>
+    <mergeCell ref="D42:F42"/>
+    <mergeCell ref="D58:F58"/>
+    <mergeCell ref="D71:F71"/>
+    <mergeCell ref="D84:F84"/>
+    <mergeCell ref="D100:F100"/>
+    <mergeCell ref="Q15:S15"/>
+    <mergeCell ref="A19:B21"/>
+    <mergeCell ref="E28:G28"/>
+    <mergeCell ref="C19:C21"/>
+    <mergeCell ref="D19:D21"/>
+    <mergeCell ref="E19:E21"/>
+    <mergeCell ref="F19:F21"/>
+    <mergeCell ref="G19:G21"/>
+    <mergeCell ref="T19:T21"/>
+    <mergeCell ref="H19:J19"/>
+    <mergeCell ref="H20:J20"/>
+    <mergeCell ref="H28:J28"/>
+    <mergeCell ref="K19:M19"/>
+    <mergeCell ref="K20:M20"/>
+    <mergeCell ref="K28:M28"/>
     <mergeCell ref="D113:F113"/>
     <mergeCell ref="A117:T118"/>
     <mergeCell ref="A120:T123"/>
@@ -9064,30 +8969,125 @@
     <mergeCell ref="N15:P15"/>
     <mergeCell ref="Q6:S6"/>
     <mergeCell ref="Q7:S7"/>
-    <mergeCell ref="A2:T2"/>
-    <mergeCell ref="A3:T3"/>
-    <mergeCell ref="D16:F16"/>
-    <mergeCell ref="D29:F29"/>
-    <mergeCell ref="D42:F42"/>
-    <mergeCell ref="D58:F58"/>
-    <mergeCell ref="D71:F71"/>
-    <mergeCell ref="D84:F84"/>
-    <mergeCell ref="D100:F100"/>
-    <mergeCell ref="Q15:S15"/>
-    <mergeCell ref="A19:B21"/>
-    <mergeCell ref="E28:G28"/>
-    <mergeCell ref="C19:C21"/>
-    <mergeCell ref="D19:D21"/>
-    <mergeCell ref="E19:E21"/>
-    <mergeCell ref="F19:F21"/>
-    <mergeCell ref="G19:G21"/>
-    <mergeCell ref="T19:T21"/>
-    <mergeCell ref="H19:J19"/>
-    <mergeCell ref="H20:J20"/>
-    <mergeCell ref="H28:J28"/>
-    <mergeCell ref="K19:M19"/>
-    <mergeCell ref="K20:M20"/>
-    <mergeCell ref="K28:M28"/>
+    <mergeCell ref="N19:P19"/>
+    <mergeCell ref="N20:P20"/>
+    <mergeCell ref="N28:P28"/>
+    <mergeCell ref="Q19:S19"/>
+    <mergeCell ref="Q20:S20"/>
+    <mergeCell ref="Q28:S28"/>
+    <mergeCell ref="A32:B34"/>
+    <mergeCell ref="E41:G41"/>
+    <mergeCell ref="C32:C34"/>
+    <mergeCell ref="D32:D34"/>
+    <mergeCell ref="E32:E34"/>
+    <mergeCell ref="F32:F34"/>
+    <mergeCell ref="G32:G34"/>
+    <mergeCell ref="T32:T34"/>
+    <mergeCell ref="H32:J32"/>
+    <mergeCell ref="H33:J33"/>
+    <mergeCell ref="H41:J41"/>
+    <mergeCell ref="K32:M32"/>
+    <mergeCell ref="K33:M33"/>
+    <mergeCell ref="K41:M41"/>
+    <mergeCell ref="N32:P32"/>
+    <mergeCell ref="N33:P33"/>
+    <mergeCell ref="N41:P41"/>
+    <mergeCell ref="Q32:S32"/>
+    <mergeCell ref="Q33:S33"/>
+    <mergeCell ref="Q41:S41"/>
+    <mergeCell ref="A48:B50"/>
+    <mergeCell ref="E57:G57"/>
+    <mergeCell ref="C48:C50"/>
+    <mergeCell ref="D48:D50"/>
+    <mergeCell ref="E48:E50"/>
+    <mergeCell ref="F48:F50"/>
+    <mergeCell ref="G48:G50"/>
+    <mergeCell ref="T48:T50"/>
+    <mergeCell ref="H48:J48"/>
+    <mergeCell ref="H49:J49"/>
+    <mergeCell ref="H57:J57"/>
+    <mergeCell ref="K48:M48"/>
+    <mergeCell ref="K49:M49"/>
+    <mergeCell ref="K57:M57"/>
+    <mergeCell ref="N48:P48"/>
+    <mergeCell ref="N49:P49"/>
+    <mergeCell ref="N57:P57"/>
+    <mergeCell ref="Q48:S48"/>
+    <mergeCell ref="Q49:S49"/>
+    <mergeCell ref="Q57:S57"/>
+    <mergeCell ref="A61:B63"/>
+    <mergeCell ref="E70:G70"/>
+    <mergeCell ref="C61:C63"/>
+    <mergeCell ref="D61:D63"/>
+    <mergeCell ref="E61:E63"/>
+    <mergeCell ref="F61:F63"/>
+    <mergeCell ref="G61:G63"/>
+    <mergeCell ref="T61:T63"/>
+    <mergeCell ref="H61:J61"/>
+    <mergeCell ref="H62:J62"/>
+    <mergeCell ref="H70:J70"/>
+    <mergeCell ref="K61:M61"/>
+    <mergeCell ref="K62:M62"/>
+    <mergeCell ref="K70:M70"/>
+    <mergeCell ref="N61:P61"/>
+    <mergeCell ref="N62:P62"/>
+    <mergeCell ref="N70:P70"/>
+    <mergeCell ref="Q61:S61"/>
+    <mergeCell ref="Q62:S62"/>
+    <mergeCell ref="Q70:S70"/>
+    <mergeCell ref="A74:B76"/>
+    <mergeCell ref="E83:G83"/>
+    <mergeCell ref="C74:C76"/>
+    <mergeCell ref="D74:D76"/>
+    <mergeCell ref="E74:E76"/>
+    <mergeCell ref="F74:F76"/>
+    <mergeCell ref="G74:G76"/>
+    <mergeCell ref="T74:T76"/>
+    <mergeCell ref="H74:J74"/>
+    <mergeCell ref="H75:J75"/>
+    <mergeCell ref="H83:J83"/>
+    <mergeCell ref="K74:M74"/>
+    <mergeCell ref="K75:M75"/>
+    <mergeCell ref="K83:M83"/>
+    <mergeCell ref="N74:P74"/>
+    <mergeCell ref="N75:P75"/>
+    <mergeCell ref="N83:P83"/>
+    <mergeCell ref="Q74:S74"/>
+    <mergeCell ref="Q75:S75"/>
+    <mergeCell ref="Q83:S83"/>
+    <mergeCell ref="A90:B92"/>
+    <mergeCell ref="E99:G99"/>
+    <mergeCell ref="C90:C92"/>
+    <mergeCell ref="D90:D92"/>
+    <mergeCell ref="E90:E92"/>
+    <mergeCell ref="F90:F92"/>
+    <mergeCell ref="G90:G92"/>
+    <mergeCell ref="T90:T92"/>
+    <mergeCell ref="H90:J90"/>
+    <mergeCell ref="H91:J91"/>
+    <mergeCell ref="H99:J99"/>
+    <mergeCell ref="K90:M90"/>
+    <mergeCell ref="K91:M91"/>
+    <mergeCell ref="K99:M99"/>
+    <mergeCell ref="N90:P90"/>
+    <mergeCell ref="N91:P91"/>
+    <mergeCell ref="N99:P99"/>
+    <mergeCell ref="Q90:S90"/>
+    <mergeCell ref="Q91:S91"/>
+    <mergeCell ref="Q99:S99"/>
+    <mergeCell ref="K103:M103"/>
+    <mergeCell ref="K104:M104"/>
+    <mergeCell ref="K112:M112"/>
+    <mergeCell ref="A103:B105"/>
+    <mergeCell ref="E112:G112"/>
+    <mergeCell ref="C103:C105"/>
+    <mergeCell ref="D103:D105"/>
+    <mergeCell ref="E103:E105"/>
+    <mergeCell ref="F103:F105"/>
+    <mergeCell ref="G103:G105"/>
+    <mergeCell ref="H103:J103"/>
+    <mergeCell ref="H104:J104"/>
+    <mergeCell ref="H112:J112"/>
   </mergeCells>
   <pageMargins left="0.39369999999999999" right="0.39369999999999999" top="1.0236000000000001" bottom="0.66930000000000001" header="0.39369999999999999" footer="0.39369999999999999"/>
   <pageSetup paperSize="9" scale="82" orientation="portrait" r:id="rId1"/>
@@ -9130,19 +9130,19 @@
       <c r="A2" s="55" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="35"/>
-      <c r="C2" s="35"/>
-      <c r="D2" s="35"/>
-      <c r="E2" s="35"/>
+      <c r="B2" s="48"/>
+      <c r="C2" s="48"/>
+      <c r="D2" s="48"/>
+      <c r="E2" s="48"/>
     </row>
     <row r="3" spans="1:5" ht="25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="56" t="s">
         <v>81</v>
       </c>
-      <c r="B3" s="35"/>
-      <c r="C3" s="35"/>
-      <c r="D3" s="35"/>
-      <c r="E3" s="35"/>
+      <c r="B3" s="48"/>
+      <c r="C3" s="48"/>
+      <c r="D3" s="48"/>
+      <c r="E3" s="48"/>
     </row>
     <row r="4" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
@@ -11356,9 +11356,9 @@
       <c r="A138" s="56" t="s">
         <v>190</v>
       </c>
-      <c r="B138" s="35"/>
-      <c r="C138" s="35"/>
-      <c r="D138" s="35"/>
+      <c r="B138" s="48"/>
+      <c r="C138" s="48"/>
+      <c r="D138" s="48"/>
     </row>
     <row r="139" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A139" t="s">

</xml_diff>